<commit_message>
catégotie obligatoire + màj options catégorie
</commit_message>
<xml_diff>
--- a/fichiers_test_numerotation/poules_numerotees.xlsx
+++ b/fichiers_test_numerotation/poules_numerotees.xlsx
@@ -438,13 +438,13 @@
         <v>A</v>
       </c>
       <c r="D2" t="str">
-        <v>SAINT ANDRE DE LA MARCHE BASKET-1</v>
+        <v>POITEVINIERE LE PIN-1</v>
       </c>
       <c r="E2" t="str">
-        <v>PDL0049170</v>
+        <v>PDL0049084</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -458,13 +458,13 @@
         <v>A</v>
       </c>
       <c r="D3" t="str">
-        <v>GARENNES LOIRE BASKET CLUB 49-1</v>
+        <v>SAINT ANDRE DE LA MARCHE BASKET-1</v>
       </c>
       <c r="E3" t="str">
-        <v>PDL0049126</v>
+        <v>PDL0049170</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -478,13 +478,13 @@
         <v>A</v>
       </c>
       <c r="D4" t="str">
-        <v>SPORTING CLUB BEAUCOUZE BASKET-1</v>
+        <v>GARENNES LOIRE BASKET CLUB 49-1</v>
       </c>
       <c r="E4" t="str">
-        <v>PDL0049152</v>
+        <v>PDL0049126</v>
       </c>
       <c r="F4">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -498,13 +498,13 @@
         <v>A</v>
       </c>
       <c r="D5" t="str">
-        <v>POITEVINIERE LE PIN-1</v>
+        <v>SPORTING CLUB BEAUCOUZE BASKET-1</v>
       </c>
       <c r="E5" t="str">
-        <v>PDL0049084</v>
+        <v>PDL0049152</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -558,10 +558,10 @@
         <v>A</v>
       </c>
       <c r="D8" t="str">
-        <v>ESSJ GREZ NEUVILLE-1</v>
+        <v>ANDARD BRAIN-2</v>
       </c>
       <c r="E8" t="str">
-        <v>PDL0049061</v>
+        <v>PDL0049004</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -578,10 +578,10 @@
         <v>A</v>
       </c>
       <c r="D9" t="str">
-        <v>POITEVINIERE LE PIN-3</v>
+        <v>VALLEE BASKET CLUB-8</v>
       </c>
       <c r="E9" t="str">
-        <v>PDL0049084</v>
+        <v>PDL0049117</v>
       </c>
       <c r="F9">
         <v>2</v>
@@ -598,10 +598,10 @@
         <v>A</v>
       </c>
       <c r="D10" t="str">
-        <v>CHALONNES SUR LOIRE BASKET-4</v>
+        <v>SAINTE GEMMES SUR LOIRE-1</v>
       </c>
       <c r="E10" t="str">
-        <v>PDL0049031</v>
+        <v>PDL0049143</v>
       </c>
       <c r="F10">
         <v>3</v>
@@ -618,10 +618,10 @@
         <v>A</v>
       </c>
       <c r="D11" t="str">
-        <v>SPORTING CLUB BEAUCOUZE BASKET-2</v>
+        <v>CHAMP SUR LAYON USND-1</v>
       </c>
       <c r="E11" t="str">
-        <v>PDL0049152</v>
+        <v>PDL0049032</v>
       </c>
       <c r="F11">
         <v>4</v>
@@ -638,10 +638,10 @@
         <v>A</v>
       </c>
       <c r="D12" t="str">
-        <v>SAINTE GEMMES SUR LOIRE-1</v>
+        <v>ELAN LIGÉRIEN BASKET-2</v>
       </c>
       <c r="E12" t="str">
-        <v>PDL0049143</v>
+        <v>PDL0049115</v>
       </c>
       <c r="F12">
         <v>5</v>
@@ -658,10 +658,10 @@
         <v>A</v>
       </c>
       <c r="D13" t="str">
-        <v>ELAN LIGÉRIEN BASKET-2</v>
+        <v>ESSJ GREZ NEUVILLE-1</v>
       </c>
       <c r="E13" t="str">
-        <v>PDL0049115</v>
+        <v>PDL0049061</v>
       </c>
       <c r="F13">
         <v>6</v>
@@ -678,13 +678,13 @@
         <v>B</v>
       </c>
       <c r="D14" t="str">
-        <v>PUY SAINT BONNET BASKET-1</v>
+        <v>CHOLET JF-1</v>
       </c>
       <c r="E14" t="str">
-        <v>PDL0049093</v>
+        <v>PDL0049045</v>
       </c>
       <c r="F14">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -698,10 +698,10 @@
         <v>B</v>
       </c>
       <c r="D15" t="str">
-        <v>SAINT CHRISTOPHE DU BOIS - ESSOR CHRISTOPHORIEN BASKET-1</v>
+        <v>MAULEVRIER-1</v>
       </c>
       <c r="E15" t="str">
-        <v>PDL0049097</v>
+        <v>PDL0049074</v>
       </c>
       <c r="F15">
         <v>2</v>
@@ -718,13 +718,13 @@
         <v>B</v>
       </c>
       <c r="D16" t="str">
-        <v>LA TESSOUALLE-1</v>
+        <v>SAINT CHRISTOPHE DU BOIS - ESSOR CHRISTOPHORIEN BASKET-1</v>
       </c>
       <c r="E16" t="str">
-        <v>PDL0049124</v>
+        <v>PDL0049097</v>
       </c>
       <c r="F16">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -738,13 +738,13 @@
         <v>B</v>
       </c>
       <c r="D17" t="str">
-        <v>MAULEVRIER-1</v>
+        <v>PUY SAINT BONNET BASKET-1</v>
       </c>
       <c r="E17" t="str">
-        <v>PDL0049074</v>
+        <v>PDL0049093</v>
       </c>
       <c r="F17">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18">
@@ -758,13 +758,13 @@
         <v>B</v>
       </c>
       <c r="D18" t="str">
-        <v>CHALONNES SUR LOIRE BASKET-5</v>
+        <v>LA TESSOUALLE-1</v>
       </c>
       <c r="E18" t="str">
-        <v>PDL0049031</v>
+        <v>PDL0049124</v>
       </c>
       <c r="F18">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
@@ -778,13 +778,13 @@
         <v>B</v>
       </c>
       <c r="D19" t="str">
-        <v>CTC ANDREA MACAIROIS BASKET​-1</v>
+        <v>CHOLET BASKET-3</v>
       </c>
       <c r="E19" t="str">
-        <v>PDL0049170</v>
+        <v>PDL0049043</v>
       </c>
       <c r="F19">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -798,13 +798,13 @@
         <v>C</v>
       </c>
       <c r="D20" t="str">
-        <v>VAL HYROME BASKET-1</v>
+        <v>CORON/SALLE DE VIHIERS-1</v>
       </c>
       <c r="E20" t="str">
-        <v>PDL0049027</v>
+        <v>PDL0049050</v>
       </c>
       <c r="F20">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -818,13 +818,13 @@
         <v>C</v>
       </c>
       <c r="D21" t="str">
-        <v>GARENNES LOIRE BASKET CLUB 49-2</v>
+        <v>JUB JALLAIS BASKET-1</v>
       </c>
       <c r="E21" t="str">
-        <v>PDL0049126</v>
+        <v>PDL0049063</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -838,13 +838,13 @@
         <v>C</v>
       </c>
       <c r="D22" t="str">
-        <v>CHALONNES SUR LOIRE BASKET-2</v>
+        <v>VAL HYROME BASKET-1</v>
       </c>
       <c r="E22" t="str">
-        <v>PDL0049031</v>
+        <v>PDL0049027</v>
       </c>
       <c r="F22">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -864,7 +864,7 @@
         <v>PDL0049084</v>
       </c>
       <c r="F23">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
@@ -878,13 +878,13 @@
         <v>C</v>
       </c>
       <c r="D24" t="str">
-        <v>SAINT ANDRE DE LA MARCHE BASKET-2</v>
+        <v>CTC ANDREA MACAIROIS BASKET​-1</v>
       </c>
       <c r="E24" t="str">
         <v>PDL0049170</v>
       </c>
       <c r="F24">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25">
@@ -898,13 +898,13 @@
         <v>C</v>
       </c>
       <c r="D25" t="str">
-        <v>ELAN LIGÉRIEN BASKET-3</v>
+        <v>BASKET LA GAULOISE LA CHAPELLE ROUSSELIN-1</v>
       </c>
       <c r="E25" t="str">
-        <v>PDL0049115</v>
+        <v>PDL0049036</v>
       </c>
       <c r="F25">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -938,7 +938,7 @@
         <v>A</v>
       </c>
       <c r="D27" t="str">
-        <v>CTC LOIRE ET PLAINE BASKET​-1</v>
+        <v>ETOILE ANGERS BASKET-2</v>
       </c>
       <c r="E27" t="str">
         <v>PDL0049095</v>
@@ -958,13 +958,13 @@
         <v>A</v>
       </c>
       <c r="D28" t="str">
-        <v>SPORTING CLUB BEAUCOUZE BASKET-3</v>
+        <v>AVRILLE BASKET-1</v>
       </c>
       <c r="E28" t="str">
-        <v>PDL0049152</v>
+        <v>PDL0049012</v>
       </c>
       <c r="F28">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
@@ -978,13 +978,13 @@
         <v>A</v>
       </c>
       <c r="D29" t="str">
-        <v>CHALONNES SUR LOIRE BASKET-3</v>
+        <v>CANDE LOIRE BASKET-1</v>
       </c>
       <c r="E29" t="str">
-        <v>PDL0049031</v>
+        <v>PDL0049077</v>
       </c>
       <c r="F29">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
@@ -1038,13 +1038,13 @@
         <v>B</v>
       </c>
       <c r="D32" t="str">
-        <v>ROSIERS-1</v>
+        <v>BRISSAC AUBANCE BASKET-1</v>
       </c>
       <c r="E32" t="str">
-        <v>PDL0049149</v>
+        <v>PDL0049024</v>
       </c>
       <c r="F32">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -1058,13 +1058,13 @@
         <v>B</v>
       </c>
       <c r="D33" t="str">
-        <v>DOUE LA FONTAINE-1</v>
+        <v>CTC LOIRE ET PLAINE BASKET​-1</v>
       </c>
       <c r="E33" t="str">
-        <v>PDL0049054</v>
+        <v>PDL0049095</v>
       </c>
       <c r="F33">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -1078,13 +1078,13 @@
         <v>B</v>
       </c>
       <c r="D34" t="str">
-        <v>BRISSAC AUBANCE BASKET-1</v>
+        <v>ROSIERS-1</v>
       </c>
       <c r="E34" t="str">
-        <v>PDL0049024</v>
+        <v>PDL0049149</v>
       </c>
       <c r="F34">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
@@ -1098,13 +1098,13 @@
         <v>B</v>
       </c>
       <c r="D35" t="str">
-        <v>ETOILE ANGERS BASKET-1</v>
+        <v>DOUE LA FONTAINE-1</v>
       </c>
       <c r="E35" t="str">
-        <v>PDL0049095</v>
+        <v>PDL0049054</v>
       </c>
       <c r="F35">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36">
@@ -1158,13 +1158,13 @@
         <v>C</v>
       </c>
       <c r="D38" t="str">
-        <v>ETRICHE BASKET-1</v>
+        <v>ANGERS ALJF-2</v>
       </c>
       <c r="E38" t="str">
-        <v>PDL0049055</v>
+        <v>PDL0049006</v>
       </c>
       <c r="F38">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -1198,13 +1198,13 @@
         <v>C</v>
       </c>
       <c r="D40" t="str">
-        <v>AVRILLE BASKET-1</v>
+        <v>ETRICHE BASKET-1</v>
       </c>
       <c r="E40" t="str">
-        <v>PDL0049012</v>
+        <v>PDL0049055</v>
       </c>
       <c r="F40">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41">
@@ -1218,13 +1218,13 @@
         <v>C</v>
       </c>
       <c r="D41" t="str">
-        <v>CTC LOIRE ET PLAINE BASKET​-2</v>
+        <v>CHAMPIGNE-3</v>
       </c>
       <c r="E41" t="str">
-        <v>PDL0049095</v>
+        <v>PDL0049033</v>
       </c>
       <c r="F41">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42">
@@ -1238,13 +1238,13 @@
         <v>C</v>
       </c>
       <c r="D42" t="str">
-        <v>ANGERS ALJF-2</v>
+        <v>CTC LOIRE ET PLAINE BASKET​-2</v>
       </c>
       <c r="E42" t="str">
-        <v>PDL0049006</v>
+        <v>PDL0049095</v>
       </c>
       <c r="F42">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43">
@@ -1298,10 +1298,10 @@
         <v>D</v>
       </c>
       <c r="D45" t="str">
-        <v>SAINT CHRISTOPHE DU BOIS - ESSOR CHRISTOPHORIEN BASKET-1</v>
+        <v>AVENIR TREMENTINES-2</v>
       </c>
       <c r="E45" t="str">
-        <v>PDL0049097</v>
+        <v>PDL0049131</v>
       </c>
       <c r="F45">
         <v>2</v>
@@ -1318,10 +1318,10 @@
         <v>D</v>
       </c>
       <c r="D46" t="str">
-        <v>SAINT ANDRE DE LA MARCHE BASKET-3</v>
+        <v>SAINT CHRISTOPHE DU BOIS - ESSOR CHRISTOPHORIEN BASKET-1</v>
       </c>
       <c r="E46" t="str">
-        <v>PDL0049170</v>
+        <v>PDL0049097</v>
       </c>
       <c r="F46">
         <v>3</v>
@@ -1338,10 +1338,10 @@
         <v>D</v>
       </c>
       <c r="D47" t="str">
-        <v>AVENIR TREMENTINES-2</v>
+        <v>TOURMELAY-1</v>
       </c>
       <c r="E47" t="str">
-        <v>PDL0049131</v>
+        <v>PDL0049128</v>
       </c>
       <c r="F47">
         <v>4</v>
@@ -1358,7 +1358,7 @@
         <v>D</v>
       </c>
       <c r="D48" t="str">
-        <v>ETOILE ANGERS BASKET-2</v>
+        <v>ETOILE ANGERS BASKET-1</v>
       </c>
       <c r="E48" t="str">
         <v>PDL0049095</v>

</xml_diff>